<commit_message>
refactor: Enhance BitacoraService with structured auditing and update dependent services
- Refactored BitacoraService to use structured columns (entidad, entidad_id, detalle) instead of JSONB for new records
- Introduced ACCIONES_VALIDAS catalog for auditable actions (LOGIN_FALLIDO, ELIMINACION, CAMBIO_ROL, ANULACION_VENTA, AJUSTE_STOCK, BAJA_STOCK, CAMBIO_PRECIO, FUSION_PRODUCTO)
- Added get_by_entidad method to retrieve audit history for specific entities
- Updated BodegasService to support es
</commit_message>
<xml_diff>
--- a/assets/downloads/productos_export.xlsx
+++ b/assets/downloads/productos_export.xlsx
@@ -424,38 +424,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="5" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>codigo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>descripcion</t>
-        </is>
-      </c>
       <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>sku</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>precio</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
@@ -472,38 +460,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>codigo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>descripcion</t>
-        </is>
-      </c>
       <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>sku</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>precio</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
@@ -512,23 +488,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>F-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Perfume Floral 100ml</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Fragancia floral</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>PF-001</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>25000</v>
-      </c>
-      <c r="E2" t="n">
+      <c r="C2" t="n">
         <v>15</v>
       </c>
     </row>

</xml_diff>